<commit_message>
feat: actualizar contenido de registro de IA
</commit_message>
<xml_diff>
--- a/Lab4_20220229_Registro_IA.xlsx
+++ b/Lab4_20220229_Registro_IA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\iot\iot_lab4_20220229\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE71AB06-2C72-42A7-AE35-8C58A2D6867B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F2C6FFB-11EC-406A-B9CF-8E8717C32870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66EF677B-24AB-4CE4-8C7B-C6293A0144E6}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>Modelo</t>
   </si>
@@ -77,13 +77,16 @@
   </si>
   <si>
     <t>“Genera una estructura óptima de archivos para un laboratorio Android con RecyclerView, Fragmentos y Navigation Component usando únicamente tecnologías vistas en clase. En formato .MD”</t>
+  </si>
+  <si>
+    <t>Registro de uso de IA para el Laboratorio 4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,6 +102,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -108,7 +119,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -131,17 +142,109 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -151,17 +254,163 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -172,6 +421,18 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{917D9689-69EA-4355-8DA7-C73C44688C55}" name="Tabla1" displayName="Tabla1" ref="B3:D8" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
+  <autoFilter ref="B3:D8" xr:uid="{917D9689-69EA-4355-8DA7-C73C44688C55}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{A852D9C5-FCD8-4097-8498-63FF9B185A5D}" name="Modelo" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{77330064-7A32-45D2-8DA8-4A8236FDC9A8}" name="Prompt" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{30DDC3A1-99B6-471D-B997-01ADE33E8802}" name="Descripción del uso de la respuesta" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -471,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02F63330-5372-456C-964E-2417B2AFE514}">
-  <dimension ref="B3:F12"/>
+  <dimension ref="B1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.88671875" customWidth="1"/>
@@ -479,113 +740,126 @@
     <col min="4" max="4" width="43.44140625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="6"/>
+    </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="2:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="2:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="2:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="2:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="2:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="2:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" spans="2:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="2:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="2:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="B8" s="7" t="s">
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="2:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B8" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="8"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="8"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="8"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:C1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>